<commit_message>
ref tracking: count unique players (dedupe by device), pay bonus on that
Raw ref_plays counts sessions, so one person replaying inflates it. Now the
play POST from every game (pitcher/batter/baller/striker/keeper/cfb) sends the
device pl_guestId, and the server records distinct (ref, uid) in a new
ref_users table -> refStats reports 'players' (unique devices/accounts) as the
creator-bonus basis alongside raw 'plays'. Docs updated: intern brief + tracker
sheet now read $10 per 1,000 new players (each person counted once); CLAUDE.md
notes the unique-player mechanism.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TYQcygZ4S9m3hBwpGw1hv9
</commit_message>
<xml_diff>
--- a/marketing/GoatLab-Creator-Tracker.xlsx
+++ b/marketing/GoatLab-Creator-Tracker.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>New users</t>
+          <t>New players</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
@@ -8753,7 +8753,7 @@
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>•  $20 for every 1,000 new users your creators send us (tracked through the links — mostly YouTube, X, Twitch).</t>
+          <t>•  $10 for every 1,000 new players your creators send us — each person counted once, not raw plays (tracked through the links — mostly YouTube, X, Twitch).</t>
         </is>
       </c>
     </row>
@@ -9105,7 +9105,7 @@
     <row r="11" ht="15" customHeight="1">
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>•  New users = the number from the tracking-link report (ask [owner] for it); it drives the $20/1,000 bonus.</t>
+          <t>•  New players = unique people from the tracking-link report, each counted once no matter how many times they play (ask [owner] for it); drives the $10/1,000 bonus.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
marketing: drop $ estimates from tracker; have intern ask creator rates
Remove the heuristic Est. rate column from the Javin-facing sheet (kept in
creator-targets.md for internal reference); add a blank 'Rate (their quote)'
column. Brief + templates now instruct: don't quote a price, ask the creator
their rate, log it, owner approves before committing.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TYQcygZ4S9m3hBwpGw1hv9
</commit_message>
<xml_diff>
--- a/marketing/GoatLab-Creator-Tracker.xlsx
+++ b/marketing/GoatLab-Creator-Tracker.xlsx
@@ -543,19 +543,19 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="26" customWidth="1" min="18" max="18"/>
   </cols>
@@ -617,22 +617,22 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Est. rate</t>
+          <t>Ref code</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Ref code</t>
+          <t>Outreach date</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Outreach date</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Rate (their quote)</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
@@ -707,11 +707,7 @@
           <t>Ratings-prediction content overlaps directly with a ratings-built game</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Dedicated ~$400–1k; integration ~$150–350 (est.)</t>
-        </is>
-      </c>
+      <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="7" t="inlineStr"/>
       <c r="K4" s="7" t="inlineStr"/>
       <c r="L4" s="7" t="inlineStr"/>
@@ -763,11 +759,7 @@
           <t>Already builds/sims player careers on camera (RTTS); GoatLab is that loop as a free browser game</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>RTTS integration ~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="7" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr"/>
       <c r="L5" s="7" t="inlineStr"/>
@@ -819,11 +811,7 @@
           <t>"Simulate a whole weird career" is his content shape</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Free seed first; ~$50–150 paid</t>
-        </is>
-      </c>
+      <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="7" t="inlineStr"/>
       <c r="K6" s="7" t="inlineStr"/>
       <c r="L6" s="7" t="inlineStr"/>
@@ -875,11 +863,7 @@
           <t>Purple Legend cards map to his nostalgia audience; high reply engagement</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Free seeding or ~$100–250 paid</t>
-        </is>
-      </c>
+      <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="7" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
@@ -931,11 +915,7 @@
           <t>Does player-rating debates — "build the perfect pitcher" is native content</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>$900–2,750 (est.)</t>
-        </is>
-      </c>
+      <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="7" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
       <c r="L8" s="7" t="inlineStr"/>
@@ -987,11 +967,7 @@
           <t>Recent MLB player; simulating his own career card is a natural video</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>$700–1,750 (est.)</t>
-        </is>
-      </c>
+      <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="7" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
@@ -1043,11 +1019,7 @@
           <t>Team-agnostic national MLB-fan reach (Legend cards); cheap</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>~$300–1k (est.)</t>
-        </is>
-      </c>
+      <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="7" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr"/>
@@ -1099,11 +1071,7 @@
           <t>Engaged skills micro audience; batter mode ties in</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>~$500–1.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="7" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr"/>
@@ -1155,11 +1123,7 @@
           <t>Velo/command/break attributes map 1:1 to his content — "building the perfect pitcher" riff</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>$500–1,250 (est.)</t>
-        </is>
-      </c>
+      <c r="I12" s="7" t="inlineStr"/>
       <c r="J12" s="7" t="inlineStr"/>
       <c r="K12" s="7" t="inlineStr"/>
       <c r="L12" s="7" t="inlineStr"/>
@@ -1211,11 +1175,7 @@
           <t>Exactly the crowd that argues about slot weights</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>Free seeding (engages with community projects)</t>
-        </is>
-      </c>
+      <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="7" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr"/>
       <c r="L13" s="7" t="inlineStr"/>
@@ -1267,11 +1227,7 @@
           <t>News format makes a "check out this game" segment natural</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$750–1.9k (est.)</t>
-        </is>
-      </c>
+      <c r="I14" s="7" t="inlineStr"/>
       <c r="J14" s="7" t="inlineStr"/>
       <c r="K14" s="7" t="inlineStr"/>
       <c r="L14" s="7" t="inlineStr"/>
@@ -1323,11 +1279,7 @@
           <t>Daily-game share culture = our core acquisition target; cross-promo partner</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>Free seeding / partnership (Sports Reference-owned)</t>
-        </is>
-      </c>
+      <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="7" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr"/>
       <c r="L15" s="7" t="inlineStr"/>
@@ -1379,11 +1331,7 @@
           <t>Interviews every creator on this list — one cheap spot + network effects into the whole niche</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>Podcast spot ~$150–600 (est.)</t>
-        </is>
-      </c>
+      <c r="I16" s="7" t="inlineStr"/>
       <c r="J16" s="7" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr"/>
       <c r="L16" s="7" t="inlineStr"/>
@@ -1435,11 +1383,7 @@
           <t>Data-driven pitching nerds map onto "build a pitcher"; cheap for the engagement</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Sponsor ~$200–800 (est.)</t>
-        </is>
-      </c>
+      <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="7" t="inlineStr"/>
       <c r="K17" s="7" t="inlineStr"/>
       <c r="L17" s="7" t="inlineStr"/>
@@ -1491,11 +1435,7 @@
           <t>Core Show ratings audience; affordable</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>Sponsored stream ~$300–900 (est.)</t>
-        </is>
-      </c>
+      <c r="I18" s="7" t="inlineStr"/>
       <c r="J18" s="7" t="inlineStr"/>
       <c r="K18" s="7" t="inlineStr"/>
       <c r="L18" s="7" t="inlineStr"/>
@@ -1547,11 +1487,7 @@
           <t>Entire brand is pitcher ratings/rankings</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>Paid ~$50–200 or content swap</t>
-        </is>
-      </c>
+      <c r="I19" s="7" t="inlineStr"/>
       <c r="J19" s="7" t="inlineStr"/>
       <c r="K19" s="7" t="inlineStr"/>
       <c r="L19" s="7" t="inlineStr"/>
@@ -1603,11 +1539,7 @@
           <t>Most pitcher-obsessed account on X; famously boosts pitching content he likes</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>Free seeding ("build Skenes' slider onto your guy" angle)</t>
-        </is>
-      </c>
+      <c r="I20" s="7" t="inlineStr"/>
       <c r="J20" s="7" t="inlineStr"/>
       <c r="K20" s="7" t="inlineStr"/>
       <c r="L20" s="7" t="inlineStr"/>
@@ -1659,11 +1591,7 @@
           <t>Ran the SDS-backed $5k Scann Community Series — ideal partner for a GoatLab build-off</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$500–1.5k (est., pending count)</t>
-        </is>
-      </c>
+      <c r="I21" s="7" t="inlineStr"/>
       <c r="J21" s="7" t="inlineStr"/>
       <c r="K21" s="7" t="inlineStr"/>
       <c r="L21" s="7" t="inlineStr"/>
@@ -1715,11 +1643,7 @@
           <t>"Create a player, watch his career" narrative = literally our premise</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>Dedicated ~$500–1.5k; TikTok ~$300–800 (est.)</t>
-        </is>
-      </c>
+      <c r="I22" s="7" t="inlineStr"/>
       <c r="J22" s="7" t="inlineStr"/>
       <c r="K22" s="7" t="inlineStr"/>
       <c r="L22" s="7" t="inlineStr"/>
@@ -1771,11 +1695,7 @@
           <t>Utility site every DD player uses daily — banner/newsletter sponsorship at utility CPMs</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>Site/video sponsorship ~$500–2k (est., negotiate direct)</t>
-        </is>
-      </c>
+      <c r="I23" s="7" t="inlineStr"/>
       <c r="J23" s="7" t="inlineStr"/>
       <c r="K23" s="7" t="inlineStr"/>
       <c r="L23" s="7" t="inlineStr"/>
@@ -1827,11 +1747,7 @@
           <t>Beloved funny pitcher persona; audience = terminally online baseball people; cheap high-engagement test buy</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>$270–675 (est.)</t>
-        </is>
-      </c>
+      <c r="I24" s="7" t="inlineStr"/>
       <c r="J24" s="7" t="inlineStr"/>
       <c r="K24" s="7" t="inlineStr"/>
       <c r="L24" s="7" t="inlineStr"/>
@@ -1883,11 +1799,7 @@
           <t>Baseball-culture comedy audience overlapping casual browser-game players</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>$900–2,600 (est.)</t>
-        </is>
-      </c>
+      <c r="I25" s="7" t="inlineStr"/>
       <c r="J25" s="7" t="inlineStr"/>
       <c r="K25" s="7" t="inlineStr"/>
       <c r="L25" s="7" t="inlineStr"/>
@@ -1939,11 +1851,7 @@
           <t>Loyal older-fan audience; modest views = realistic indie pricing</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$650–1.6k — price off views, not subs (est.)</t>
-        </is>
-      </c>
+      <c r="I26" s="7" t="inlineStr"/>
       <c r="J26" s="7" t="inlineStr"/>
       <c r="K26" s="7" t="inlineStr"/>
       <c r="L26" s="7" t="inlineStr"/>
@@ -1995,11 +1903,7 @@
           <t>#1 Show streamer by Twitch engagement — one sponsored segment reaches the hardest-core audience</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>Stream sponsorship ~$800–2.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I27" s="7" t="inlineStr"/>
       <c r="J27" s="7" t="inlineStr"/>
       <c r="K27" s="7" t="inlineStr"/>
       <c r="L27" s="7" t="inlineStr"/>
@@ -2051,11 +1955,7 @@
           <t>Small, hyper-engaged meme audience; OVR debates are his lane</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>X post ~$400–900 (est.)</t>
-        </is>
-      </c>
+      <c r="I28" s="7" t="inlineStr"/>
       <c r="J28" s="7" t="inlineStr"/>
       <c r="K28" s="7" t="inlineStr"/>
       <c r="L28" s="7" t="inlineStr"/>
@@ -2107,11 +2007,7 @@
           <t>Analytics-minded fans enjoy rating mechanics; affordable</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>Post/integration ~$800–2k (est.)</t>
-        </is>
-      </c>
+      <c r="I29" s="7" t="inlineStr"/>
       <c r="J29" s="7" t="inlineStr"/>
       <c r="K29" s="7" t="inlineStr"/>
       <c r="L29" s="7" t="inlineStr"/>
@@ -2163,11 +2059,7 @@
           <t>Ball-knowledge/ratings audience loves min-maxing a 99 OVR; cheap</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>Cross-post ~$700–1.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I30" s="7" t="inlineStr"/>
       <c r="J30" s="7" t="inlineStr"/>
       <c r="K30" s="7" t="inlineStr"/>
       <c r="L30" s="7" t="inlineStr"/>
@@ -2219,11 +2111,7 @@
           <t>Near-perfect match; his audience literally watches "how to build a player"</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>Dedicated ~$500–1.3k (est.)</t>
-        </is>
-      </c>
+      <c r="I31" s="7" t="inlineStr"/>
       <c r="J31" s="7" t="inlineStr"/>
       <c r="K31" s="7" t="inlineStr"/>
       <c r="L31" s="7" t="inlineStr"/>
@@ -2275,11 +2163,7 @@
           <t>Builds/rebuilds rosters from real ratings; near-identical mechanic</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$500–1.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I32" s="7" t="inlineStr"/>
       <c r="J32" s="7" t="inlineStr"/>
       <c r="K32" s="7" t="inlineStr"/>
       <c r="L32" s="7" t="inlineStr"/>
@@ -2331,11 +2215,7 @@
           <t>Short-form CFB takes audience; indie-friendly self-monetizing creator</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>$1.5k–3.8k/TikTok (est.)</t>
-        </is>
-      </c>
+      <c r="I33" s="7" t="inlineStr"/>
       <c r="J33" s="7" t="inlineStr"/>
       <c r="K33" s="7" t="inlineStr"/>
       <c r="L33" s="7" t="inlineStr"/>
@@ -2387,11 +2267,7 @@
           <t>Faceless meme pages charge far below personal-creator rates; pure CFB-fan firehose</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>$250–1k/post (est., unverified)</t>
-        </is>
-      </c>
+      <c r="I34" s="7" t="inlineStr"/>
       <c r="J34" s="7" t="inlineStr"/>
       <c r="K34" s="7" t="inlineStr"/>
       <c r="L34" s="7" t="inlineStr"/>
@@ -2443,11 +2319,7 @@
           <t>Hardcore CFB stat nerds who will min-max a ratings game; dedicated video fits budget</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>$900–2,250 dedicated (est.)</t>
-        </is>
-      </c>
+      <c r="I35" s="7" t="inlineStr"/>
       <c r="J35" s="7" t="inlineStr"/>
       <c r="K35" s="7" t="inlineStr"/>
       <c r="L35" s="7" t="inlineStr"/>
@@ -2499,11 +2371,7 @@
           <t>Career-mode / create-a-player content is the closest match; EA-vetted</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>~$800–2.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I36" s="7" t="inlineStr"/>
       <c r="J36" s="7" t="inlineStr"/>
       <c r="K36" s="7" t="inlineStr"/>
       <c r="L36" s="7" t="inlineStr"/>
@@ -2555,11 +2423,7 @@
           <t>CFB comedy audience; Signing Day / mascot flavor is on-brand</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>~$1.7k–5k (est.)</t>
-        </is>
-      </c>
+      <c r="I37" s="7" t="inlineStr"/>
       <c r="J37" s="7" t="inlineStr"/>
       <c r="K37" s="7" t="inlineStr"/>
       <c r="L37" s="7" t="inlineStr"/>
@@ -2611,11 +2475,7 @@
           <t>Affordable, multi-platform, plays a lot of EA CFB on stream</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>~$800–2.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I38" s="7" t="inlineStr"/>
       <c r="J38" s="7" t="inlineStr"/>
       <c r="K38" s="7" t="inlineStr"/>
       <c r="L38" s="7" t="inlineStr"/>
@@ -2667,11 +2527,7 @@
           <t>Cheap high-velocity CFB reach; tracked-link post fits</t>
         </is>
       </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>~$600–1.8k (est.)</t>
-        </is>
-      </c>
+      <c r="I39" s="7" t="inlineStr"/>
       <c r="J39" s="7" t="inlineStr"/>
       <c r="K39" s="7" t="inlineStr"/>
       <c r="L39" s="7" t="inlineStr"/>
@@ -2723,11 +2579,7 @@
           <t>Dynasty superfan audience; easy live "build-a-QB" segment</t>
         </is>
       </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>Stream segment ~$300–1k (est.)</t>
-        </is>
-      </c>
+      <c r="I40" s="7" t="inlineStr"/>
       <c r="J40" s="7" t="inlineStr"/>
       <c r="K40" s="7" t="inlineStr"/>
       <c r="L40" s="7" t="inlineStr"/>
@@ -2779,11 +2631,7 @@
           <t>Affordable engaged mid audience; playful build-video format</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k; mention ~$500–1.2k (est.)</t>
-        </is>
-      </c>
+      <c r="I41" s="7" t="inlineStr"/>
       <c r="J41" s="7" t="inlineStr"/>
       <c r="K41" s="7" t="inlineStr"/>
       <c r="L41" s="7" t="inlineStr"/>
@@ -2835,11 +2683,7 @@
           <t>Audience is natively about player ratings/cards; cheap X post</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>~$500–1.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I42" s="7" t="inlineStr"/>
       <c r="J42" s="7" t="inlineStr"/>
       <c r="K42" s="7" t="inlineStr"/>
       <c r="L42" s="7" t="inlineStr"/>
@@ -2891,11 +2735,7 @@
           <t>Micro meme reach at near-throwaway cost</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>~$300–900 (est.)</t>
-        </is>
-      </c>
+      <c r="I43" s="7" t="inlineStr"/>
       <c r="J43" s="7" t="inlineStr"/>
       <c r="K43" s="7" t="inlineStr"/>
       <c r="L43" s="7" t="inlineStr"/>
@@ -2947,11 +2787,7 @@
           <t>Closest content match; pioneered EA NHL YouTube</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>Dedicated ~$3k–8k; integration ~$1k–2.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I44" s="7" t="inlineStr"/>
       <c r="J44" s="7" t="inlineStr"/>
       <c r="K44" s="7" t="inlineStr"/>
       <c r="L44" s="7" t="inlineStr"/>
@@ -3003,11 +2839,7 @@
           <t>Meme accounts drive cheap viral reach; "build a 99" is meme-able</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>~$1k–3k; story ~$400–900 (est.)</t>
-        </is>
-      </c>
+      <c r="I45" s="7" t="inlineStr"/>
       <c r="J45" s="7" t="inlineStr"/>
       <c r="K45" s="7" t="inlineStr"/>
       <c r="L45" s="7" t="inlineStr"/>
@@ -3059,11 +2891,7 @@
           <t>Micro, cheap, tight hockey-comedy niche; ideal indie test</t>
         </is>
       </c>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>~$300–850 (est.)</t>
-        </is>
-      </c>
+      <c r="I46" s="7" t="inlineStr"/>
       <c r="J46" s="7" t="inlineStr"/>
       <c r="K46" s="7" t="inlineStr"/>
       <c r="L46" s="7" t="inlineStr"/>
@@ -3115,11 +2943,7 @@
           <t>Direct gameplay match; cheap native live segment</t>
         </is>
       </c>
-      <c r="I47" s="6" t="inlineStr">
-        <is>
-          <t>Stream segment ~$150–600 (est.)</t>
-        </is>
-      </c>
+      <c r="I47" s="7" t="inlineStr"/>
       <c r="J47" s="7" t="inlineStr"/>
       <c r="K47" s="7" t="inlineStr"/>
       <c r="L47" s="7" t="inlineStr"/>
@@ -3171,11 +2995,7 @@
           <t>Owner pick; playful "spin your guy" reaction format. Email: drewfennytv@gmail.com</t>
         </is>
       </c>
-      <c r="I48" s="6" t="inlineStr">
-        <is>
-          <t>~$650–1.6k (est.)</t>
-        </is>
-      </c>
+      <c r="I48" s="7" t="inlineStr"/>
       <c r="J48" s="7" t="inlineStr"/>
       <c r="K48" s="7" t="inlineStr"/>
       <c r="L48" s="7" t="inlineStr"/>
@@ -3227,11 +3047,7 @@
           <t>Spans several GoatLab modes at once; native fit for a live "spin &amp; build" segment</t>
         </is>
       </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>Stream segment ~$300–1k (est.)</t>
-        </is>
-      </c>
+      <c r="I49" s="7" t="inlineStr"/>
       <c r="J49" s="7" t="inlineStr"/>
       <c r="K49" s="7" t="inlineStr"/>
       <c r="L49" s="7" t="inlineStr"/>
@@ -3283,11 +3099,7 @@
           <t>True micro, cheap, hyper-engaged FM niche; ideal test buy</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>~$100–500 (est.)</t>
-        </is>
-      </c>
+      <c r="I50" s="7" t="inlineStr"/>
       <c r="J50" s="7" t="inlineStr"/>
       <c r="K50" s="7" t="inlineStr"/>
       <c r="L50" s="7" t="inlineStr"/>
@@ -3339,11 +3151,7 @@
           <t>Longest-running FM series; loves player-progression hooks</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I51" s="7" t="inlineStr"/>
       <c r="J51" s="7" t="inlineStr"/>
       <c r="K51" s="7" t="inlineStr"/>
       <c r="L51" s="7" t="inlineStr"/>
@@ -3395,11 +3203,7 @@
           <t>FM "build a wonderkid" audience overlaps directly</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$1.5k–3k (est.)</t>
-        </is>
-      </c>
+      <c r="I52" s="7" t="inlineStr"/>
       <c r="J52" s="7" t="inlineStr"/>
       <c r="K52" s="7" t="inlineStr"/>
       <c r="L52" s="7" t="inlineStr"/>
@@ -3451,11 +3255,7 @@
           <t>Niche engaged FM fanbase, affordable, sim-native</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$1k–2.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I53" s="7" t="inlineStr"/>
       <c r="J53" s="7" t="inlineStr"/>
       <c r="K53" s="7" t="inlineStr"/>
       <c r="L53" s="7" t="inlineStr"/>
@@ -3507,11 +3307,7 @@
           <t>American FM creator; closest content match (build-a-club sim), US-reachable</t>
         </is>
       </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>Integration ~$2k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I54" s="7" t="inlineStr"/>
       <c r="J54" s="7" t="inlineStr"/>
       <c r="K54" s="7" t="inlineStr"/>
       <c r="L54" s="7" t="inlineStr"/>
@@ -3563,11 +3359,7 @@
           <t>Pure baseball-comedy reach at mid-tier pricing</t>
         </is>
       </c>
-      <c r="I55" s="11" t="inlineStr">
-        <is>
-          <t>$4.4k–13.3k (est.)</t>
-        </is>
-      </c>
+      <c r="I55" s="7" t="inlineStr"/>
       <c r="J55" s="7" t="inlineStr"/>
       <c r="K55" s="7" t="inlineStr"/>
       <c r="L55" s="7" t="inlineStr"/>
@@ -3619,11 +3411,7 @@
           <t>Broad MLB meme/highlight audience; shareable clips</t>
         </is>
       </c>
-      <c r="I56" s="8" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I56" s="7" t="inlineStr"/>
       <c r="J56" s="7" t="inlineStr"/>
       <c r="K56" s="7" t="inlineStr"/>
       <c r="L56" s="7" t="inlineStr"/>
@@ -3675,11 +3463,7 @@
           <t>Engaged skills audience; batter crossover</t>
         </is>
       </c>
-      <c r="I57" s="11" t="inlineStr">
-        <is>
-          <t>~$700–2k (est.)</t>
-        </is>
-      </c>
+      <c r="I57" s="7" t="inlineStr"/>
       <c r="J57" s="7" t="inlineStr"/>
       <c r="K57" s="7" t="inlineStr"/>
       <c r="L57" s="7" t="inlineStr"/>
@@ -3731,11 +3515,7 @@
           <t>Verified active; confirm size before outreach</t>
         </is>
       </c>
-      <c r="I58" s="8" t="inlineStr">
-        <is>
-          <t>Free seeding</t>
-        </is>
-      </c>
+      <c r="I58" s="7" t="inlineStr"/>
       <c r="J58" s="7" t="inlineStr"/>
       <c r="K58" s="7" t="inlineStr"/>
       <c r="L58" s="7" t="inlineStr"/>
@@ -3787,11 +3567,7 @@
           <t>Casual baseball-fan crowd; matches a lightweight game</t>
         </is>
       </c>
-      <c r="I59" s="11" t="inlineStr">
-        <is>
-          <t>~$1k–3k (est.)</t>
-        </is>
-      </c>
+      <c r="I59" s="7" t="inlineStr"/>
       <c r="J59" s="7" t="inlineStr"/>
       <c r="K59" s="7" t="inlineStr"/>
       <c r="L59" s="7" t="inlineStr"/>
@@ -3843,11 +3619,7 @@
           <t>Collector audience overlaps with collect/rate mechanic; cheap</t>
         </is>
       </c>
-      <c r="I60" s="8" t="inlineStr">
-        <is>
-          <t>~$300–800 (est.)</t>
-        </is>
-      </c>
+      <c r="I60" s="7" t="inlineStr"/>
       <c r="J60" s="7" t="inlineStr"/>
       <c r="K60" s="7" t="inlineStr"/>
       <c r="L60" s="7" t="inlineStr"/>
@@ -3899,11 +3671,7 @@
           <t>Audience = players who'd share OVR builds</t>
         </is>
       </c>
-      <c r="I61" s="11" t="inlineStr">
-        <is>
-          <t>$2.5k–7.6k (est.)</t>
-        </is>
-      </c>
+      <c r="I61" s="7" t="inlineStr"/>
       <c r="J61" s="7" t="inlineStr"/>
       <c r="K61" s="7" t="inlineStr"/>
       <c r="L61" s="7" t="inlineStr"/>
@@ -3955,11 +3723,7 @@
           <t>Big casual baseball-culture reach; playful tone</t>
         </is>
       </c>
-      <c r="I62" s="8" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I62" s="7" t="inlineStr"/>
       <c r="J62" s="7" t="inlineStr"/>
       <c r="K62" s="7" t="inlineStr"/>
       <c r="L62" s="7" t="inlineStr"/>
@@ -4011,11 +3775,7 @@
           <t>Meme-fluent audience, engages with fan-made stuff</t>
         </is>
       </c>
-      <c r="I63" s="11" t="inlineStr">
-        <is>
-          <t>Free seed; ~$300–500 shoutout</t>
-        </is>
-      </c>
+      <c r="I63" s="7" t="inlineStr"/>
       <c r="J63" s="7" t="inlineStr"/>
       <c r="K63" s="7" t="inlineStr"/>
       <c r="L63" s="7" t="inlineStr"/>
@@ -4067,11 +3827,7 @@
           <t>Career-card screenshots made for their QT culture</t>
         </is>
       </c>
-      <c r="I64" s="8" t="inlineStr">
-        <is>
-          <t>Paid (network rates); tag in seeding regardless</t>
-        </is>
-      </c>
+      <c r="I64" s="7" t="inlineStr"/>
       <c r="J64" s="7" t="inlineStr"/>
       <c r="K64" s="7" t="inlineStr"/>
       <c r="L64" s="7" t="inlineStr"/>
@@ -4123,11 +3879,7 @@
           <t>Community favorite for funny casual content; goofy browser game suits him</t>
         </is>
       </c>
-      <c r="I65" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$1.9k–4.8k (est.)</t>
-        </is>
-      </c>
+      <c r="I65" s="7" t="inlineStr"/>
       <c r="J65" s="7" t="inlineStr"/>
       <c r="K65" s="7" t="inlineStr"/>
       <c r="L65" s="7" t="inlineStr"/>
@@ -4179,11 +3931,7 @@
           <t>High-frequency DD machine, always needs fresh baseball-game material</t>
         </is>
       </c>
-      <c r="I66" s="8" t="inlineStr">
-        <is>
-          <t>Integration ~$1.9k–4.7k (est.)</t>
-        </is>
-      </c>
+      <c r="I66" s="7" t="inlineStr"/>
       <c r="J66" s="7" t="inlineStr"/>
       <c r="K66" s="7" t="inlineStr"/>
       <c r="L66" s="7" t="inlineStr"/>
@@ -4235,11 +3983,7 @@
           <t>Baseball-obsessed play-the-game crowd</t>
         </is>
       </c>
-      <c r="I67" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$3.5k–8k (est.)</t>
-        </is>
-      </c>
+      <c r="I67" s="7" t="inlineStr"/>
       <c r="J67" s="7" t="inlineStr"/>
       <c r="K67" s="7" t="inlineStr"/>
       <c r="L67" s="7" t="inlineStr"/>
@@ -4291,11 +4035,7 @@
           <t>Sim diehards who love stat lines + HOF verdicts</t>
         </is>
       </c>
-      <c r="I68" s="8" t="inlineStr">
-        <is>
-          <t>Dedicated ~$150–600 (est.)</t>
-        </is>
-      </c>
+      <c r="I68" s="7" t="inlineStr"/>
       <c r="J68" s="7" t="inlineStr"/>
       <c r="K68" s="7" t="inlineStr"/>
       <c r="L68" s="7" t="inlineStr"/>
@@ -4347,11 +4087,7 @@
           <t>The single most on-brand account in baseball for this game</t>
         </is>
       </c>
-      <c r="I69" s="11" t="inlineStr">
-        <is>
-          <t>$3.5k–10.5k (est.; not a typical sponsor account — seed free first)</t>
-        </is>
-      </c>
+      <c r="I69" s="7" t="inlineStr"/>
       <c r="J69" s="7" t="inlineStr"/>
       <c r="K69" s="7" t="inlineStr"/>
       <c r="L69" s="7" t="inlineStr"/>
@@ -4403,11 +4139,7 @@
           <t>10-yr pro explaining pitching — perfect demo for slot-by-slot builds</t>
         </is>
       </c>
-      <c r="I70" s="8" t="inlineStr">
-        <is>
-          <t>$3.9k–11.8k (est.)</t>
-        </is>
-      </c>
+      <c r="I70" s="7" t="inlineStr"/>
       <c r="J70" s="7" t="inlineStr"/>
       <c r="K70" s="7" t="inlineStr"/>
       <c r="L70" s="7" t="inlineStr"/>
@@ -4459,11 +4191,7 @@
           <t>Provably sponsorable (official MiLB IronPigs deal)</t>
         </is>
       </c>
-      <c r="I71" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$1.3k–3.3k (est.)</t>
-        </is>
-      </c>
+      <c r="I71" s="7" t="inlineStr"/>
       <c r="J71" s="7" t="inlineStr"/>
       <c r="K71" s="7" t="inlineStr"/>
       <c r="L71" s="7" t="inlineStr"/>
@@ -4515,11 +4243,7 @@
           <t>Their audience plays exactly these share-your-result games</t>
         </is>
       </c>
-      <c r="I72" s="8" t="inlineStr">
-        <is>
-          <t>Seed free; paid via Jomboy sales ($500+)</t>
-        </is>
-      </c>
+      <c r="I72" s="7" t="inlineStr"/>
       <c r="J72" s="7" t="inlineStr"/>
       <c r="K72" s="7" t="inlineStr"/>
       <c r="L72" s="7" t="inlineStr"/>
@@ -4571,11 +4295,7 @@
           <t>Large casual crowd; pricier, less gaming-focused</t>
         </is>
       </c>
-      <c r="I73" s="11" t="inlineStr">
-        <is>
-          <t>~$2k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I73" s="7" t="inlineStr"/>
       <c r="J73" s="7" t="inlineStr"/>
       <c r="K73" s="7" t="inlineStr"/>
       <c r="L73" s="7" t="inlineStr"/>
@@ -4627,11 +4347,7 @@
           <t>High-authority hitting audience for batter mode</t>
         </is>
       </c>
-      <c r="I74" s="8" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I74" s="7" t="inlineStr"/>
       <c r="J74" s="7" t="inlineStr"/>
       <c r="K74" s="7" t="inlineStr"/>
       <c r="L74" s="7" t="inlineStr"/>
@@ -4683,11 +4399,7 @@
           <t>Skills audience, mid and affordable</t>
         </is>
       </c>
-      <c r="I75" s="11" t="inlineStr">
-        <is>
-          <t>~$600–1.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I75" s="7" t="inlineStr"/>
       <c r="J75" s="7" t="inlineStr"/>
       <c r="K75" s="7" t="inlineStr"/>
       <c r="L75" s="7" t="inlineStr"/>
@@ -4739,11 +4451,7 @@
           <t>Serious pitching audience; may prefer a brand deal</t>
         </is>
       </c>
-      <c r="I76" s="8" t="inlineStr">
-        <is>
-          <t>~$2k–5k (est.)</t>
-        </is>
-      </c>
+      <c r="I76" s="7" t="inlineStr"/>
       <c r="J76" s="7" t="inlineStr"/>
       <c r="K76" s="7" t="inlineStr"/>
       <c r="L76" s="7" t="inlineStr"/>
@@ -4795,11 +4503,7 @@
           <t>Indie data-viz project beloved by Baseball Twitter</t>
         </is>
       </c>
-      <c r="I77" s="11" t="inlineStr">
-        <is>
-          <t>Free seeding; contact creator</t>
-        </is>
-      </c>
+      <c r="I77" s="7" t="inlineStr"/>
       <c r="J77" s="7" t="inlineStr"/>
       <c r="K77" s="7" t="inlineStr"/>
       <c r="L77" s="7" t="inlineStr"/>
@@ -4851,11 +4555,7 @@
           <t>Proof indie baseball web tools go viral here; indie-builder peer</t>
         </is>
       </c>
-      <c r="I78" s="8" t="inlineStr">
-        <is>
-          <t>Free seeding (peer-to-peer angle)</t>
-        </is>
-      </c>
+      <c r="I78" s="7" t="inlineStr"/>
       <c r="J78" s="7" t="inlineStr"/>
       <c r="K78" s="7" t="inlineStr"/>
       <c r="L78" s="7" t="inlineStr"/>
@@ -4907,11 +4607,7 @@
           <t>Tier-list format overlaps with "assign a rating"; bracket audience</t>
         </is>
       </c>
-      <c r="I79" s="11" t="inlineStr">
-        <is>
-          <t>TikTok ~$3k–7k; X cheaper (est.)</t>
-        </is>
-      </c>
+      <c r="I79" s="7" t="inlineStr"/>
       <c r="J79" s="7" t="inlineStr"/>
       <c r="K79" s="7" t="inlineStr"/>
       <c r="L79" s="7" t="inlineStr"/>
@@ -4963,11 +4659,7 @@
           <t>2K pack-opening audience = the slot-machine reel mechanic</t>
         </is>
       </c>
-      <c r="I80" s="8" t="inlineStr">
-        <is>
-          <t>Integration ~$6k–15k (est.)</t>
-        </is>
-      </c>
+      <c r="I80" s="7" t="inlineStr"/>
       <c r="J80" s="7" t="inlineStr"/>
       <c r="K80" s="7" t="inlineStr"/>
       <c r="L80" s="7" t="inlineStr"/>
@@ -5019,11 +4711,7 @@
           <t>Core 2K MyPlayer audience; "build a 99" challenge fits</t>
         </is>
       </c>
-      <c r="I81" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$8k–20k (est.)</t>
-        </is>
-      </c>
+      <c r="I81" s="7" t="inlineStr"/>
       <c r="J81" s="7" t="inlineStr"/>
       <c r="K81" s="7" t="inlineStr"/>
       <c r="L81" s="7" t="inlineStr"/>
@@ -5075,11 +4763,7 @@
           <t>Stats/rating-literate viewers; fun segment potential</t>
         </is>
       </c>
-      <c r="I82" s="8" t="inlineStr">
-        <is>
-          <t>Integration ~$12k–25k (est.)</t>
-        </is>
-      </c>
+      <c r="I82" s="7" t="inlineStr"/>
       <c r="J82" s="7" t="inlineStr"/>
       <c r="K82" s="7" t="inlineStr"/>
       <c r="L82" s="7" t="inlineStr"/>
@@ -5131,11 +4815,7 @@
           <t>Broad NBA-gaming crossover; casual free game fits</t>
         </is>
       </c>
-      <c r="I83" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$8k–18k (est.)</t>
-        </is>
-      </c>
+      <c r="I83" s="7" t="inlineStr"/>
       <c r="J83" s="7" t="inlineStr"/>
       <c r="K83" s="7" t="inlineStr"/>
       <c r="L83" s="7" t="inlineStr"/>
@@ -5187,11 +4867,7 @@
           <t>Big NBA-Twitter distribution for a tracked-link post</t>
         </is>
       </c>
-      <c r="I84" s="8" t="inlineStr">
-        <is>
-          <t>~$2k–5k (est.)</t>
-        </is>
-      </c>
+      <c r="I84" s="7" t="inlineStr"/>
       <c r="J84" s="7" t="inlineStr"/>
       <c r="K84" s="7" t="inlineStr"/>
       <c r="L84" s="7" t="inlineStr"/>
@@ -5243,11 +4919,7 @@
           <t>Massive viral NBA-Twitter reach; funny "build" post fits</t>
         </is>
       </c>
-      <c r="I85" s="11" t="inlineStr">
-        <is>
-          <t>~$2.5k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I85" s="7" t="inlineStr"/>
       <c r="J85" s="7" t="inlineStr"/>
       <c r="K85" s="7" t="inlineStr"/>
       <c r="L85" s="7" t="inlineStr"/>
@@ -5299,11 +4971,7 @@
           <t>Broad CFB reach via one sponsored post</t>
         </is>
       </c>
-      <c r="I86" s="8" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I86" s="7" t="inlineStr"/>
       <c r="J86" s="7" t="inlineStr"/>
       <c r="K86" s="7" t="inlineStr"/>
       <c r="L86" s="7" t="inlineStr"/>
@@ -5355,11 +5023,7 @@
           <t>Perfect content overlap; big engaged CFB-gaming base</t>
         </is>
       </c>
-      <c r="I87" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I87" s="7" t="inlineStr"/>
       <c r="J87" s="7" t="inlineStr"/>
       <c r="K87" s="7" t="inlineStr"/>
       <c r="L87" s="7" t="inlineStr"/>
@@ -5411,11 +5075,7 @@
           <t>Most influential CFB-rebuild creator; his anger at EA CFB27 microtransactions makes a FREE browser CFB game a perfect counter-narrative pitch</t>
         </is>
       </c>
-      <c r="I88" s="8" t="inlineStr">
-        <is>
-          <t>Dedicated $12k–30k; short/integration $5k–14k (est.)</t>
-        </is>
-      </c>
+      <c r="I88" s="7" t="inlineStr"/>
       <c r="J88" s="7" t="inlineStr"/>
       <c r="K88" s="7" t="inlineStr"/>
       <c r="L88" s="7" t="inlineStr"/>
@@ -5467,11 +5127,7 @@
           <t>Simple sponsored shoutout to a pure-CFB audience</t>
         </is>
       </c>
-      <c r="I89" s="11" t="inlineStr">
-        <is>
-          <t>~$800–2k (est.)</t>
-        </is>
-      </c>
+      <c r="I89" s="7" t="inlineStr"/>
       <c r="J89" s="7" t="inlineStr"/>
       <c r="K89" s="7" t="inlineStr"/>
       <c r="L89" s="7" t="inlineStr"/>
@@ -5523,11 +5179,7 @@
           <t>Our Signing Day hat-grab IS his format — "commit graphic for your simulated player" gag</t>
         </is>
       </c>
-      <c r="I90" s="8" t="inlineStr">
-        <is>
-          <t>$4k–10k/post (est.; On3 employment may complicate)</t>
-        </is>
-      </c>
+      <c r="I90" s="7" t="inlineStr"/>
       <c r="J90" s="7" t="inlineStr"/>
       <c r="K90" s="7" t="inlineStr"/>
       <c r="L90" s="7" t="inlineStr"/>
@@ -5579,11 +5231,7 @@
           <t>His "brutally honest college career" humor = our verdict tiers ("Hall of Walk-Ons")</t>
         </is>
       </c>
-      <c r="I91" s="11" t="inlineStr">
-        <is>
-          <t>TBD after size check</t>
-        </is>
-      </c>
+      <c r="I91" s="7" t="inlineStr"/>
       <c r="J91" s="7" t="inlineStr"/>
       <c r="K91" s="7" t="inlineStr"/>
       <c r="L91" s="7" t="inlineStr"/>
@@ -5635,11 +5283,7 @@
           <t>Beloved CFB brand; "build your recruit" sketch would resonate</t>
         </is>
       </c>
-      <c r="I92" s="8" t="inlineStr">
-        <is>
-          <t>Branded sketch ~$2k–5k (est.)</t>
-        </is>
-      </c>
+      <c r="I92" s="7" t="inlineStr"/>
       <c r="J92" s="7" t="inlineStr"/>
       <c r="K92" s="7" t="inlineStr"/>
       <c r="L92" s="7" t="inlineStr"/>
@@ -5691,11 +5335,7 @@
           <t>High-engagement CFB comedy; rivalry angle suits team-picking</t>
         </is>
       </c>
-      <c r="I93" s="11" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I93" s="7" t="inlineStr"/>
       <c r="J93" s="7" t="inlineStr"/>
       <c r="K93" s="7" t="inlineStr"/>
       <c r="L93" s="7" t="inlineStr"/>
@@ -5747,11 +5387,7 @@
           <t>Nostalgic for old NCAA games, critical of EA — receptive to an indie alternative</t>
         </is>
       </c>
-      <c r="I94" s="8" t="inlineStr">
-        <is>
-          <t>Dedicated $3.5k–8.5k; mention $1k–2k (est.)</t>
-        </is>
-      </c>
+      <c r="I94" s="7" t="inlineStr"/>
       <c r="J94" s="7" t="inlineStr"/>
       <c r="K94" s="7" t="inlineStr"/>
       <c r="L94" s="7" t="inlineStr"/>
@@ -5803,11 +5439,7 @@
           <t>NFL-fan comedy; affordable on IG/TikTok</t>
         </is>
       </c>
-      <c r="I95" s="11" t="inlineStr">
-        <is>
-          <t>~$800–2k (est.)</t>
-        </is>
-      </c>
+      <c r="I95" s="7" t="inlineStr"/>
       <c r="J95" s="7" t="inlineStr"/>
       <c r="K95" s="7" t="inlineStr"/>
       <c r="L95" s="7" t="inlineStr"/>
@@ -5859,11 +5491,7 @@
           <t>Already narrates RTG careers episode-by-episode</t>
         </is>
       </c>
-      <c r="I96" s="8" t="inlineStr">
-        <is>
-          <t>TBD after size check</t>
-        </is>
-      </c>
+      <c r="I96" s="7" t="inlineStr"/>
       <c r="J96" s="7" t="inlineStr"/>
       <c r="K96" s="7" t="inlineStr"/>
       <c r="L96" s="7" t="inlineStr"/>
@@ -5915,11 +5543,7 @@
           <t>Big multi-platform hockey-gamer audience</t>
         </is>
       </c>
-      <c r="I97" s="11" t="inlineStr">
-        <is>
-          <t>Dedicated ~$2.5k–6k; integration ~$800–2k (est.)</t>
-        </is>
-      </c>
+      <c r="I97" s="7" t="inlineStr"/>
       <c r="J97" s="7" t="inlineStr"/>
       <c r="K97" s="7" t="inlineStr"/>
       <c r="L97" s="7" t="inlineStr"/>
@@ -5971,11 +5595,7 @@
           <t>Mid TikTok reach, affordable</t>
         </is>
       </c>
-      <c r="I98" s="8" t="inlineStr">
-        <is>
-          <t>~$1.2k–3.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I98" s="7" t="inlineStr"/>
       <c r="J98" s="7" t="inlineStr"/>
       <c r="K98" s="7" t="inlineStr"/>
       <c r="L98" s="7" t="inlineStr"/>
@@ -6027,11 +5647,7 @@
           <t>Proven brand-deal creator, broad culture reach</t>
         </is>
       </c>
-      <c r="I99" s="11" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k; mention ~$600–1.2k (est.)</t>
-        </is>
-      </c>
+      <c r="I99" s="7" t="inlineStr"/>
       <c r="J99" s="7" t="inlineStr"/>
       <c r="K99" s="7" t="inlineStr"/>
       <c r="L99" s="7" t="inlineStr"/>
@@ -6083,11 +5699,7 @@
           <t>Deeply-hockey audience; does product/tool features</t>
         </is>
       </c>
-      <c r="I100" s="8" t="inlineStr">
-        <is>
-          <t>Dedicated ~$2k–5k; integration ~$700–1.8k (est.)</t>
-        </is>
-      </c>
+      <c r="I100" s="7" t="inlineStr"/>
       <c r="J100" s="7" t="inlineStr"/>
       <c r="K100" s="7" t="inlineStr"/>
       <c r="L100" s="7" t="inlineStr"/>
@@ -6139,11 +5751,7 @@
           <t>Large casual highlight audience; efficient IG post</t>
         </is>
       </c>
-      <c r="I101" s="11" t="inlineStr">
-        <is>
-          <t>~$1.5k–4k; story ~$600–1.2k (est.)</t>
-        </is>
-      </c>
+      <c r="I101" s="7" t="inlineStr"/>
       <c r="J101" s="7" t="inlineStr"/>
       <c r="K101" s="7" t="inlineStr"/>
       <c r="L101" s="7" t="inlineStr"/>
@@ -6195,11 +5803,7 @@
           <t>Mid engaged TikTok audience, budget-friendly</t>
         </is>
       </c>
-      <c r="I102" s="8" t="inlineStr">
-        <is>
-          <t>~$1k–3k (est.)</t>
-        </is>
-      </c>
+      <c r="I102" s="7" t="inlineStr"/>
       <c r="J102" s="7" t="inlineStr"/>
       <c r="K102" s="7" t="inlineStr"/>
       <c r="L102" s="7" t="inlineStr"/>
@@ -6251,11 +5855,7 @@
           <t>Huge casual reach; "build the perfect goalie" hook</t>
         </is>
       </c>
-      <c r="I103" s="11" t="inlineStr">
-        <is>
-          <t>Dedicated ~$2k–5k; mention ~$700–1.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I103" s="7" t="inlineStr"/>
       <c r="J103" s="7" t="inlineStr"/>
       <c r="K103" s="7" t="inlineStr"/>
       <c r="L103" s="7" t="inlineStr"/>
@@ -6307,11 +5907,7 @@
           <t>Comedy-forward hockey-Twitter reach; low-cost post</t>
         </is>
       </c>
-      <c r="I104" s="8" t="inlineStr">
-        <is>
-          <t>~$500–1.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I104" s="7" t="inlineStr"/>
       <c r="J104" s="7" t="inlineStr"/>
       <c r="K104" s="7" t="inlineStr"/>
       <c r="L104" s="7" t="inlineStr"/>
@@ -6363,11 +5959,7 @@
           <t>Rides the biggest hockey brand at a fraction of the pod price</t>
         </is>
       </c>
-      <c r="I105" s="11" t="inlineStr">
-        <is>
-          <t>~$800–2.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I105" s="7" t="inlineStr"/>
       <c r="J105" s="7" t="inlineStr"/>
       <c r="K105" s="7" t="inlineStr"/>
       <c r="L105" s="7" t="inlineStr"/>
@@ -6419,11 +6011,7 @@
           <t>Loyal fanbase; podcast read ideal for a link drop</t>
         </is>
       </c>
-      <c r="I106" s="8" t="inlineStr">
-        <is>
-          <t>Podcast read ~$1k–3k (est.)</t>
-        </is>
-      </c>
+      <c r="I106" s="7" t="inlineStr"/>
       <c r="J106" s="7" t="inlineStr"/>
       <c r="K106" s="7" t="inlineStr"/>
       <c r="L106" s="7" t="inlineStr"/>
@@ -6475,11 +6063,7 @@
           <t>Player-rating-obsessed audience; daily uploads</t>
         </is>
       </c>
-      <c r="I107" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$2.5k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I107" s="7" t="inlineStr"/>
       <c r="J107" s="7" t="inlineStr"/>
       <c r="K107" s="7" t="inlineStr"/>
       <c r="L107" s="7" t="inlineStr"/>
@@ -6531,11 +6115,7 @@
           <t>Florida-based, English, WC2026 creator correspondent</t>
         </is>
       </c>
-      <c r="I108" s="8" t="inlineStr">
-        <is>
-          <t>~$300–2k (est.)</t>
-        </is>
-      </c>
+      <c r="I108" s="7" t="inlineStr"/>
       <c r="J108" s="7" t="inlineStr"/>
       <c r="K108" s="7" t="inlineStr"/>
       <c r="L108" s="7" t="inlineStr"/>
@@ -6587,11 +6167,7 @@
           <t>Comp EA FC audience obsessed with player ratings</t>
         </is>
       </c>
-      <c r="I109" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$4k–10k (est.)</t>
-        </is>
-      </c>
+      <c r="I109" s="7" t="inlineStr"/>
       <c r="J109" s="7" t="inlineStr"/>
       <c r="K109" s="7" t="inlineStr"/>
       <c r="L109" s="7" t="inlineStr"/>
@@ -6643,11 +6219,7 @@
           <t>Huge cheap reach on X; build-screenshot content is native</t>
         </is>
       </c>
-      <c r="I110" s="8" t="inlineStr">
-        <is>
-          <t>~$1k–4k (est.)</t>
-        </is>
-      </c>
+      <c r="I110" s="7" t="inlineStr"/>
       <c r="J110" s="7" t="inlineStr"/>
       <c r="K110" s="7" t="inlineStr"/>
       <c r="L110" s="7" t="inlineStr"/>
@@ -6699,11 +6271,7 @@
           <t>Ratings / "who's better" list format maps onto build-an-OVR</t>
         </is>
       </c>
-      <c r="I111" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$3k–7k (est.)</t>
-        </is>
-      </c>
+      <c r="I111" s="7" t="inlineStr"/>
       <c r="J111" s="7" t="inlineStr"/>
       <c r="K111" s="7" t="inlineStr"/>
       <c r="L111" s="7" t="inlineStr"/>
@@ -6755,11 +6323,7 @@
           <t>Live UT audience good for a spin-and-build segment</t>
         </is>
       </c>
-      <c r="I112" s="8" t="inlineStr">
-        <is>
-          <t>Twitch segment ~$2k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I112" s="7" t="inlineStr"/>
       <c r="J112" s="7" t="inlineStr"/>
       <c r="K112" s="7" t="inlineStr"/>
       <c r="L112" s="7" t="inlineStr"/>
@@ -6811,11 +6375,7 @@
           <t>Ultimate Team teaching audience; OVR framing matches</t>
         </is>
       </c>
-      <c r="I113" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$3k–8k (est.)</t>
-        </is>
-      </c>
+      <c r="I113" s="7" t="inlineStr"/>
       <c r="J113" s="7" t="inlineStr"/>
       <c r="K113" s="7" t="inlineStr"/>
       <c r="L113" s="7" t="inlineStr"/>
@@ -6867,11 +6427,7 @@
           <t>US-based, English, broad soccer-culture reach, affordable</t>
         </is>
       </c>
-      <c r="I114" s="8" t="inlineStr">
-        <is>
-          <t>~$2k–5k (est.)</t>
-        </is>
-      </c>
+      <c r="I114" s="7" t="inlineStr"/>
       <c r="J114" s="7" t="inlineStr"/>
       <c r="K114" s="7" t="inlineStr"/>
       <c r="L114" s="7" t="inlineStr"/>
@@ -6923,11 +6479,7 @@
           <t>Micro, cheap; meme format suits a "99 OVR" screenshot</t>
         </is>
       </c>
-      <c r="I115" s="11" t="inlineStr">
-        <is>
-          <t>~$50–300 (est.)</t>
-        </is>
-      </c>
+      <c r="I115" s="7" t="inlineStr"/>
       <c r="J115" s="7" t="inlineStr"/>
       <c r="K115" s="7" t="inlineStr"/>
       <c r="L115" s="7" t="inlineStr"/>
@@ -6979,11 +6531,7 @@
           <t>Ratings/meta-savvy competitive audience; brand-friendly</t>
         </is>
       </c>
-      <c r="I116" s="8" t="inlineStr">
-        <is>
-          <t>Integration ~$2k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I116" s="7" t="inlineStr"/>
       <c r="J116" s="7" t="inlineStr"/>
       <c r="K116" s="7" t="inlineStr"/>
       <c r="L116" s="7" t="inlineStr"/>
@@ -7035,11 +6583,7 @@
           <t>Better fit for Batting Lab; equipment-focused and large</t>
         </is>
       </c>
-      <c r="I117" s="11" t="inlineStr">
-        <is>
-          <t>agency ($8k+)</t>
-        </is>
-      </c>
+      <c r="I117" s="7" t="inlineStr"/>
       <c r="J117" s="7" t="inlineStr"/>
       <c r="K117" s="7" t="inlineStr"/>
       <c r="L117" s="7" t="inlineStr"/>
@@ -7091,11 +6635,7 @@
           <t>Huge engaged reach, above the affordable band</t>
         </is>
       </c>
-      <c r="I118" s="8" t="inlineStr">
-        <is>
-          <t>~$5k–15k (est.)</t>
-        </is>
-      </c>
+      <c r="I118" s="7" t="inlineStr"/>
       <c r="J118" s="7" t="inlineStr"/>
       <c r="K118" s="7" t="inlineStr"/>
       <c r="L118" s="7" t="inlineStr"/>
@@ -7147,11 +6687,7 @@
           <t>Legacy tastemakers; RT = "Baseball Twitter approved"</t>
         </is>
       </c>
-      <c r="I119" s="11" t="inlineStr">
-        <is>
-          <t>Free seeding only (employed journalists)</t>
-        </is>
-      </c>
+      <c r="I119" s="7" t="inlineStr"/>
       <c r="J119" s="7" t="inlineStr"/>
       <c r="K119" s="7" t="inlineStr"/>
       <c r="L119" s="7" t="inlineStr"/>
@@ -7203,11 +6739,7 @@
           <t>Defining pitcher-adjacent comedy creator; priced past indie budget</t>
         </is>
       </c>
-      <c r="I120" s="8" t="inlineStr">
-        <is>
-          <t>agency ($8k–20k+)</t>
-        </is>
-      </c>
+      <c r="I120" s="7" t="inlineStr"/>
       <c r="J120" s="7" t="inlineStr"/>
       <c r="K120" s="7" t="inlineStr"/>
       <c r="L120" s="7" t="inlineStr"/>
@@ -7259,11 +6791,7 @@
           <t>Straddles real-MLB and Show audiences — the exact crossover we target</t>
         </is>
       </c>
-      <c r="I121" s="11" t="inlineStr">
-        <is>
-          <t>Dedicated ~$6k–15k; integration ~$2k–5k (est.)</t>
-        </is>
-      </c>
+      <c r="I121" s="7" t="inlineStr"/>
       <c r="J121" s="7" t="inlineStr"/>
       <c r="K121" s="7" t="inlineStr"/>
       <c r="L121" s="7" t="inlineStr"/>
@@ -7315,11 +6843,7 @@
           <t>Baseball-entertainment crossover king (Gatorade/Reebok = agency pricing)</t>
         </is>
       </c>
-      <c r="I122" s="8" t="inlineStr">
-        <is>
-          <t>agency ($10k+)</t>
-        </is>
-      </c>
+      <c r="I122" s="7" t="inlineStr"/>
       <c r="J122" s="7" t="inlineStr"/>
       <c r="K122" s="7" t="inlineStr"/>
       <c r="L122" s="7" t="inlineStr"/>
@@ -7371,11 +6895,7 @@
           <t>Only partially baseball; priced large</t>
         </is>
       </c>
-      <c r="I123" s="11" t="inlineStr">
-        <is>
-          <t>agency ($8k+)</t>
-        </is>
-      </c>
+      <c r="I123" s="7" t="inlineStr"/>
       <c r="J123" s="7" t="inlineStr"/>
       <c r="K123" s="7" t="inlineStr"/>
       <c r="L123" s="7" t="inlineStr"/>
@@ -7427,11 +6947,7 @@
           <t>Massive credibility, but MLB-invested media co = way past indie budget</t>
         </is>
       </c>
-      <c r="I124" s="8" t="inlineStr">
-        <is>
-          <t>agency-only ($15k+)</t>
-        </is>
-      </c>
+      <c r="I124" s="7" t="inlineStr"/>
       <c r="J124" s="7" t="inlineStr"/>
       <c r="K124" s="7" t="inlineStr"/>
       <c r="L124" s="7" t="inlineStr"/>
@@ -7483,11 +6999,7 @@
           <t>Ratings-literate audience that already obsesses over attribute numbers</t>
         </is>
       </c>
-      <c r="I125" s="11" t="inlineStr">
-        <is>
-          <t>Dedicated ~$8k–20k; integration ~$2.7k–6.7k (est.)</t>
-        </is>
-      </c>
+      <c r="I125" s="7" t="inlineStr"/>
       <c r="J125" s="7" t="inlineStr"/>
       <c r="K125" s="7" t="inlineStr"/>
       <c r="L125" s="7" t="inlineStr"/>
@@ -7539,11 +7051,7 @@
           <t>The biggest RTTS/career-mode channel — "build a guy and sim his career" is exactly his format</t>
         </is>
       </c>
-      <c r="I126" s="8" t="inlineStr">
-        <is>
-          <t>Dedicated ~$6.5k–16.5k; integration ~$2.2k–5.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I126" s="7" t="inlineStr"/>
       <c r="J126" s="7" t="inlineStr"/>
       <c r="K126" s="7" t="inlineStr"/>
       <c r="L126" s="7" t="inlineStr"/>
@@ -7595,11 +7103,7 @@
           <t>Challenge-style content adapts to "spin the reel" hooks</t>
         </is>
       </c>
-      <c r="I127" s="11" t="inlineStr">
-        <is>
-          <t>$2k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I127" s="7" t="inlineStr"/>
       <c r="J127" s="7" t="inlineStr"/>
       <c r="K127" s="7" t="inlineStr"/>
       <c r="L127" s="7" t="inlineStr"/>
@@ -7651,11 +7155,7 @@
           <t>Large 2K audience; macro pricing</t>
         </is>
       </c>
-      <c r="I128" s="8" t="inlineStr">
-        <is>
-          <t>Integration ~$15k–30k (est.)</t>
-        </is>
-      </c>
+      <c r="I128" s="7" t="inlineStr"/>
       <c r="J128" s="7" t="inlineStr"/>
       <c r="K128" s="7" t="inlineStr"/>
       <c r="L128" s="7" t="inlineStr"/>
@@ -7707,11 +7207,7 @@
           <t>Big hoops-gaming reach; too pricey</t>
         </is>
       </c>
-      <c r="I129" s="11" t="inlineStr">
-        <is>
-          <t>Macro/negotiated</t>
-        </is>
-      </c>
+      <c r="I129" s="7" t="inlineStr"/>
       <c r="J129" s="7" t="inlineStr"/>
       <c r="K129" s="7" t="inlineStr"/>
       <c r="L129" s="7" t="inlineStr"/>
@@ -7763,11 +7259,7 @@
           <t>Reach exists but broadcaster rates, looser fit</t>
         </is>
       </c>
-      <c r="I130" s="8" t="inlineStr">
-        <is>
-          <t>~$3k–7k (est.)</t>
-        </is>
-      </c>
+      <c r="I130" s="7" t="inlineStr"/>
       <c r="J130" s="7" t="inlineStr"/>
       <c r="K130" s="7" t="inlineStr"/>
       <c r="L130" s="7" t="inlineStr"/>
@@ -7819,11 +7311,7 @@
           <t>2K core audience; macro pricing</t>
         </is>
       </c>
-      <c r="I131" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$10k–22k (est.)</t>
-        </is>
-      </c>
+      <c r="I131" s="7" t="inlineStr"/>
       <c r="J131" s="7" t="inlineStr"/>
       <c r="K131" s="7" t="inlineStr"/>
       <c r="L131" s="7" t="inlineStr"/>
@@ -7875,11 +7363,7 @@
           <t>Broad reach, but not a ratings/gaming audience; macro</t>
         </is>
       </c>
-      <c r="I132" s="8" t="inlineStr">
-        <is>
-          <t>Macro/negotiated</t>
-        </is>
-      </c>
+      <c r="I132" s="7" t="inlineStr"/>
       <c r="J132" s="7" t="inlineStr"/>
       <c r="K132" s="7" t="inlineStr"/>
       <c r="L132" s="7" t="inlineStr"/>
@@ -7931,11 +7415,7 @@
           <t>Signature wager/challenge format maps onto build-and-sim</t>
         </is>
       </c>
-      <c r="I133" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$12k–25k (est.)</t>
-        </is>
-      </c>
+      <c r="I133" s="7" t="inlineStr"/>
       <c r="J133" s="7" t="inlineStr"/>
       <c r="K133" s="7" t="inlineStr"/>
       <c r="L133" s="7" t="inlineStr"/>
@@ -7987,11 +7467,7 @@
           <t>Huge casual reach but macro CPM</t>
         </is>
       </c>
-      <c r="I134" s="8" t="inlineStr">
-        <is>
-          <t>Macro/negotiated</t>
-        </is>
-      </c>
+      <c r="I134" s="7" t="inlineStr"/>
       <c r="J134" s="7" t="inlineStr"/>
       <c r="K134" s="7" t="inlineStr"/>
       <c r="L134" s="7" t="inlineStr"/>
@@ -8043,11 +7519,7 @@
           <t>Massive sports-comedy reach; pricey</t>
         </is>
       </c>
-      <c r="I135" s="11" t="inlineStr">
-        <is>
-          <t>~$4k–10k (est.)</t>
-        </is>
-      </c>
+      <c r="I135" s="7" t="inlineStr"/>
       <c r="J135" s="7" t="inlineStr"/>
       <c r="K135" s="7" t="inlineStr"/>
       <c r="L135" s="7" t="inlineStr"/>
@@ -8099,11 +7571,7 @@
           <t>Sponsorships route through Barstool sales, not indie DMs</t>
         </is>
       </c>
-      <c r="I136" s="8" t="inlineStr">
-        <is>
-          <t>$1.2k–3k+ (est., via Barstool)</t>
-        </is>
-      </c>
+      <c r="I136" s="7" t="inlineStr"/>
       <c r="J136" s="7" t="inlineStr"/>
       <c r="K136" s="7" t="inlineStr"/>
       <c r="L136" s="7" t="inlineStr"/>
@@ -8155,11 +7623,7 @@
           <t>Big NFL-culture reach; too costly for a lean budget</t>
         </is>
       </c>
-      <c r="I137" s="11" t="inlineStr">
-        <is>
-          <t>~$3k–8k (est.)</t>
-        </is>
-      </c>
+      <c r="I137" s="7" t="inlineStr"/>
       <c r="J137" s="7" t="inlineStr"/>
       <c r="K137" s="7" t="inlineStr"/>
       <c r="L137" s="7" t="inlineStr"/>
@@ -8211,11 +7675,7 @@
           <t>Audience opens CFB game content daily; news format = integrations only</t>
         </is>
       </c>
-      <c r="I138" s="8" t="inlineStr">
-        <is>
-          <t>Integration $2k–5k (est.)</t>
-        </is>
-      </c>
+      <c r="I138" s="7" t="inlineStr"/>
       <c r="J138" s="7" t="inlineStr"/>
       <c r="K138" s="7" t="inlineStr"/>
       <c r="L138" s="7" t="inlineStr"/>
@@ -8267,11 +7727,7 @@
           <t>Career arcs (busts, legends) map to sim verdicts — but priced far above budget</t>
         </is>
       </c>
-      <c r="I139" s="11" t="inlineStr">
-        <is>
-          <t>$18k–45k dedicated (est.)</t>
-        </is>
-      </c>
+      <c r="I139" s="7" t="inlineStr"/>
       <c r="J139" s="7" t="inlineStr"/>
       <c r="K139" s="7" t="inlineStr"/>
       <c r="L139" s="7" t="inlineStr"/>
@@ -8323,11 +7779,7 @@
           <t>Broad casual reach beyond the sim-gamer niche</t>
         </is>
       </c>
-      <c r="I140" s="8" t="inlineStr">
-        <is>
-          <t>$6k–15k/TikTok (est.)</t>
-        </is>
-      </c>
+      <c r="I140" s="7" t="inlineStr"/>
       <c r="J140" s="7" t="inlineStr"/>
       <c r="K140" s="7" t="inlineStr"/>
       <c r="L140" s="7" t="inlineStr"/>
@@ -8379,11 +7831,7 @@
           <t>Exact-audience match; larger reach, pricier</t>
         </is>
       </c>
-      <c r="I141" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$3k–6k (est.)</t>
-        </is>
-      </c>
+      <c r="I141" s="7" t="inlineStr"/>
       <c r="J141" s="7" t="inlineStr"/>
       <c r="K141" s="7" t="inlineStr"/>
       <c r="L141" s="7" t="inlineStr"/>
@@ -8435,11 +7883,7 @@
           <t>Madden reach, but MUT-heavy = looser fit</t>
         </is>
       </c>
-      <c r="I142" s="8" t="inlineStr">
-        <is>
-          <t>Integration ~$2k–4.5k (est.)</t>
-        </is>
-      </c>
+      <c r="I142" s="7" t="inlineStr"/>
       <c r="J142" s="7" t="inlineStr"/>
       <c r="K142" s="7" t="inlineStr"/>
       <c r="L142" s="7" t="inlineStr"/>
@@ -8491,11 +7935,7 @@
           <t>Enormous reach, out of budget; note for scale-up</t>
         </is>
       </c>
-      <c r="I143" s="11" t="inlineStr">
-        <is>
-          <t>~$20k–60k+ (est.)</t>
-        </is>
-      </c>
+      <c r="I143" s="7" t="inlineStr"/>
       <c r="J143" s="7" t="inlineStr"/>
       <c r="K143" s="7" t="inlineStr"/>
       <c r="L143" s="7" t="inlineStr"/>
@@ -8547,11 +7987,7 @@
           <t>Great fit but too expensive</t>
         </is>
       </c>
-      <c r="I144" s="8" t="inlineStr">
-        <is>
-          <t>~$15k–50k (est.)</t>
-        </is>
-      </c>
+      <c r="I144" s="7" t="inlineStr"/>
       <c r="J144" s="7" t="inlineStr"/>
       <c r="K144" s="7" t="inlineStr"/>
       <c r="L144" s="7" t="inlineStr"/>
@@ -8603,11 +8039,7 @@
           <t>Massive UT audience; above budget except a small integration</t>
         </is>
       </c>
-      <c r="I145" s="11" t="inlineStr">
-        <is>
-          <t>Integration ~$8k–25k (est.)</t>
-        </is>
-      </c>
+      <c r="I145" s="7" t="inlineStr"/>
       <c r="J145" s="7" t="inlineStr"/>
       <c r="K145" s="7" t="inlineStr"/>
       <c r="L145" s="7" t="inlineStr"/>
@@ -8659,11 +8091,7 @@
           <t>Analytical audience fits ratings depth but brand-owned + pricey</t>
         </is>
       </c>
-      <c r="I146" s="8" t="inlineStr">
-        <is>
-          <t>~$10k–30k (est.)</t>
-        </is>
-      </c>
+      <c r="I146" s="7" t="inlineStr"/>
       <c r="J146" s="7" t="inlineStr"/>
       <c r="K146" s="7" t="inlineStr"/>
       <c r="L146" s="7" t="inlineStr"/>
@@ -8681,7 +8109,7 @@
     <mergeCell ref="A1:R1"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="L4:L146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K4:K146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"X DM,Email,IG DM,TikTok DM,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="M4:M146" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -8707,7 +8135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8808,64 +8236,71 @@
     <row r="16" ht="15" customHeight="1">
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>•  Never say we're affiliated with MLB, MLB The Show, or EA. It's "real MLB ratings," that's it.</t>
+          <t>•  Don't quote a price to creators. Ask what their rate is, log it in the Rate column, and send it to [owner] to approve before committing to anything paid.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>•  If anyone asks, be upfront you're reaching out on behalf of GoatLab.</t>
+          <t>•  Never say we're affiliated with MLB, MLB The Show, or EA. It's "real MLB ratings," that's it.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>•  Keep it human in the DMs — a real person who likes the game, not a bot.</t>
+          <t>•  If anyone asks, be upfront you're reaching out on behalf of GoatLab.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>•  Max ~10-15 reach-outs a day per platform. One follow-up only if they ghost (5-7 days later).</t>
+          <t>•  Keep it human in the DMs — a real person who likes the game, not a bot.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="17" t="inlineStr">
         <is>
+          <t>•  Max ~10-15 reach-outs a day per platform. One follow-up only if they ghost (5-7 days later).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="B21" s="17" t="inlineStr">
+        <is>
           <t>•  Personalize the first line every time — mention a recent post/video. No copy-paste blasts.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="B21" s="17" t="inlineStr"/>
-    </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr"/>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Who to target</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>•  All sports (baseball, basketball, soccer, football) are fair game; gaming creators are a secondary lane.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>•  At least 5k followers, active in the last couple weeks, real engagement (not bots).</t>
+          <t>•  All sports (baseball, basketball, soccer, football) are fair game; gaming creators are a secondary lane.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>•  At least 5k followers, active in the last couple weeks, real engagement (not bots).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>•  Work the list on the Creators tab top-down by Priority, and add your own finds to the bottom.</t>
         </is>
@@ -8885,7 +8320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8972,50 +8407,57 @@
     <row r="14" ht="15" customHeight="1">
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Offer: $[X] for one dedicated video (or $[Y] integration + a pinned-comment Daily follow-up a week later). You'd use your tracked link goat-lab.app/?ref=[code] and I'll share the click-to-play numbers. Creative is all yours; only ask is the link in the description and saying it's free. Interested?</t>
+          <t>I'd love to sponsor a video. What's your rate for a dedicated video or an integration? You'd use your tracked link goat-lab.app/?ref=[code] and I'll share the click-to-play numbers. Creative is all yours; only ask is the link in the description and saying it's free. Interested?</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="B15" s="17" t="inlineStr"/>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>(Don't throw out a dollar number yourself — let them quote it, log it, and I'll approve.)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>3. Paid-offer terms (after they say yes)</t>
-        </is>
-      </c>
+      <c r="B16" s="17" t="inlineStr"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>•  Deliverable: [1 dedicated video / 2 posts a week apart / 1 stream segment 20+ min]</t>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>3. Paid-offer terms (after they say yes AND [owner] approves their rate)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>•  Fee: $[X], paid [50% upfront / on posting] via [Venmo/PayPal]</t>
+          <t>•  Deliverable: [1 dedicated video / 2 posts a week apart / 1 stream segment 20+ min]</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>•  Required: tracked link goat-lab.app/?ref=[code] in [description/bio/pinned comment]; mention it's free</t>
+          <t>•  Fee: their quoted rate (they name it; [owner] approves before you commit), paid [50% upfront / on posting]</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>•  Disclosure: mark it #ad/sponsored (FTC)</t>
+          <t>•  Required: tracked link goat-lab.app/?ref=[code] in [description/bio/pinned comment]; mention it's free</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>•  Disclosure: mark it #ad/sponsored (FTC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>•  Creative control fully theirs; no exclusivity</t>
         </is>

</xml_diff>

<commit_message>
marketing: use owner's cold-DM script in tracker Templates tab, strip em dashes
Replace the generic cold DM with the owner's voice (main + shorter variant);
remove em dashes across the whole workbook (templates, rules, and Creators
research text).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TYQcygZ4S9m3hBwpGw1hv9
</commit_message>
<xml_diff>
--- a/marketing/GoatLab-Creator-Tracker.xlsx
+++ b/marketing/GoatLab-Creator-Tracker.xlsx
@@ -563,7 +563,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GoatLab — Creator Outreach Tracker</t>
+          <t>GoatLab: Creator Outreach Tracker</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Does player-rating debates — "build the perfect pitcher" is native content</t>
+          <t>Does player-rating debates - "build the perfect pitcher" is native content</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr"/>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>Velo/command/break attributes map 1:1 to his content — "building the perfect pitcher" riff</t>
+          <t>Velo/command/break attributes map 1:1 to his content - "building the perfect pitcher" riff</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>Interviews every creator on this list — one cheap spot + network effects into the whole niche</t>
+          <t>Interviews every creator on this list - one cheap spot + network effects into the whole niche</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr"/>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Ran the SDS-backed $5k Scann Community Series — ideal partner for a GoatLab build-off</t>
+          <t>Ran the SDS-backed $5k Scann Community Series - ideal partner for a GoatLab build-off</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr"/>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Utility site every DD player uses daily — banner/newsletter sponsorship at utility CPMs</t>
+          <t>Utility site every DD player uses daily - banner/newsletter sponsorship at utility CPMs</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr"/>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>#1 Show streamer by Twitch engagement — one sponsored segment reaches the hardest-core audience</t>
+          <t>#1 Show streamer by Twitch engagement - one sponsored segment reaches the hardest-core audience</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr"/>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>10-yr pro explaining pitching — perfect demo for slot-by-slot builds</t>
+          <t>10-yr pro explaining pitching - perfect demo for slot-by-slot builds</t>
         </is>
       </c>
       <c r="I70" s="7" t="inlineStr"/>
@@ -5037,7 +5037,7 @@
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t>Medium (stretch — pitch integration)</t>
+          <t>Medium (stretch - pitch integration)</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="H90" s="8" t="inlineStr">
         <is>
-          <t>Our Signing Day hat-grab IS his format — "commit graphic for your simulated player" gag</t>
+          <t>Our Signing Day hat-grab IS his format - "commit graphic for your simulated player" gag</t>
         </is>
       </c>
       <c r="I90" s="7" t="inlineStr"/>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="H94" s="8" t="inlineStr">
         <is>
-          <t>Nostalgic for old NCAA games, critical of EA — receptive to an indie alternative</t>
+          <t>Nostalgic for old NCAA games, critical of EA - receptive to an indie alternative</t>
         </is>
       </c>
       <c r="I94" s="7" t="inlineStr"/>
@@ -6788,7 +6788,7 @@
       </c>
       <c r="H121" s="11" t="inlineStr">
         <is>
-          <t>Straddles real-MLB and Show audiences — the exact crossover we target</t>
+          <t>Straddles real-MLB and Show audiences - the exact crossover we target</t>
         </is>
       </c>
       <c r="I121" s="7" t="inlineStr"/>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="H126" s="8" t="inlineStr">
         <is>
-          <t>The biggest RTTS/career-mode channel — "build a guy and sim his career" is exactly his format</t>
+          <t>The biggest RTTS/career-mode channel - "build a guy and sim his career" is exactly his format</t>
         </is>
       </c>
       <c r="I126" s="7" t="inlineStr"/>
@@ -7724,7 +7724,7 @@
       </c>
       <c r="H139" s="11" t="inlineStr">
         <is>
-          <t>Career arcs (busts, legends) map to sim verdicts — but priced far above budget</t>
+          <t>Career arcs (busts, legends) map to sim verdicts - but priced far above budget</t>
         </is>
       </c>
       <c r="I139" s="7" t="inlineStr"/>
@@ -8160,7 +8160,7 @@
     <row r="4" ht="15" customHeight="1">
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>•  $50/week for the first two weeks — a trial run for both of us.</t>
+          <t>•  $50/week for the first two weeks, a trial run for both of us.</t>
         </is>
       </c>
     </row>
@@ -8181,7 +8181,7 @@
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>•  $10 for every 1,000 new players your creators send us — each person counted once, not raw plays (tracked through the links — mostly YouTube, X, Twitch).</t>
+          <t>•  $10 for every 1,000 new players your creators send us, each person counted once (not raw plays), tracked through the links (mostly YouTube, X, Twitch).</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
     <row r="13" ht="15" customHeight="1">
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>A post only counts once it's LIVE and has the tracking link in it. A shoutout with no link doesn't count — we can't track it and it barely sends anyone.</t>
+          <t>A post only counts once it's LIVE and has the tracking link in it. A shoutout with no link doesn't count, since we can't track it and it barely sends anyone.</t>
         </is>
       </c>
     </row>
@@ -8257,7 +8257,7 @@
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>•  Keep it human in the DMs — a real person who likes the game, not a bot.</t>
+          <t>•  Keep it human in the DMs, a real person who likes the game, not a bot.</t>
         </is>
       </c>
     </row>
@@ -8271,7 +8271,7 @@
     <row r="21" ht="15" customHeight="1">
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>•  Personalize the first line every time — mention a recent post/video. No copy-paste blasts.</t>
+          <t>•  Personalize the first line every time, mention a recent post/video. No copy-paste blasts.</t>
         </is>
       </c>
     </row>
@@ -8320,7 +8320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -8338,21 +8338,21 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>1. Cold DM — TikTok / Instagram / X (free seeding)</t>
+          <t>1. Cold DM (X / Instagram / TikTok) - the go-to</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="B4" s="17" t="inlineStr">
         <is>
-          <t>Hey [name] — [one specific line about a recent post of theirs]. I made a free browser game I think your audience would eat up: spin a random real [sport] player, choose where each rating goes on his body, then simulate his whole career. No download, takes 3 minutes: goat-lab.app/?ref=[code]</t>
+          <t>Hey [Name]! Love your content, [that video/post about ___] was awesome. Was wondering if you'd be down to try out my game? You spin a wheel, land on a random [baseball] player, then build the GOAT using the best attributes from the guys you get, and you can sim their whole career after. It's free and takes like 2 min: goat-lab.app/?ref=[code]</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>No ask — just thought it was your kind of thing. If you ever want to post it, the funniest format we've seen is "building the worst player possible" and reading the career verdict.</t>
+          <t>Lmk if you'd maybe be interested in making a video/post playing it! No pressure either way.</t>
         </is>
       </c>
     </row>
@@ -8362,102 +8362,126 @@
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Follow-up (once, 5-7 days later, only if no reply)</t>
+          <t>1b. Shorter version (DMs do better tight)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>One more nudge and I'll leave you alone — today's Daily Challenge gives everyone the same cards, so "beat my score" actually works on your audience: goat-lab.app/?ref=[code]</t>
+          <t>Hey [Name]! Big fan of your stuff, [that ___ video] was great. Made a free game I think you'd vibe with. You spin a wheel, land on a random [baseball] player, and build the GOAT from the best attributes, then sim the career. Takes 2 min: goat-lab.app/?ref=[code]</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="B9" s="17" t="inlineStr"/>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Lmk if you'd wanna make a video/post on it!</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>2. Email — YouTube / Twitch (paid)</t>
-        </is>
-      </c>
+      <c r="B10" s="17" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>Subject: Sponsor idea — build-a-99 browser game your audience will get instantly</t>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Follow-up (once, 5-7 days later, only if no reply)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>Hi [name], I'm with GoatLab (goat-lab.app), a free browser game where you spin real players with real ratings, assign each to a body part, build a 99 OVR, and simulate the career. I'd love to sponsor a video.</t>
+          <t>One more nudge and I'll leave you alone! Today's Daily Challenge gives everyone the same cards, so "beat my score" actually works on your audience: goat-lab.app/?ref=[code]</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Formats that work: God Squad vs Cursed Squad (best vs worst build), a 1v1 vs a viewer, or "Beat my Daily" where your audience plays the same cards.</t>
-        </is>
-      </c>
+      <c r="B13" s="17" t="inlineStr"/>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>I'd love to sponsor a video. What's your rate for a dedicated video or an integration? You'd use your tracked link goat-lab.app/?ref=[code] and I'll share the click-to-play numbers. Creative is all yours; only ask is the link in the description and saying it's free. Interested?</t>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>2. Email (YouTube / Twitch, paid)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>(Don't throw out a dollar number yourself — let them quote it, log it, and I'll approve.)</t>
+          <t>Subject: Sponsor idea: build-a-99 browser game your audience will get instantly</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="17" t="inlineStr"/>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Hi [name], I'm with GoatLab (goat-lab.app), a free browser game where you spin real players with real ratings, assign each to a body part, build a 99 OVR, and simulate the career. I'd love to sponsor a video.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>3. Paid-offer terms (after they say yes AND [owner] approves their rate)</t>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Formats that work: God Squad vs Cursed Squad (best vs worst build), a 1v1 vs a viewer, or "Beat my Daily" where your audience plays the same cards.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>•  Deliverable: [1 dedicated video / 2 posts a week apart / 1 stream segment 20+ min]</t>
+          <t>I'd love to sponsor a video. What's your rate for a dedicated video or an integration? You'd use your tracked link goat-lab.app/?ref=[code] and I'll share the click-to-play numbers. Creative is all yours; only ask is the link in the description and saying it's free. Interested?</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>•  Fee: their quoted rate (they name it; [owner] approves before you commit), paid [50% upfront / on posting]</t>
+          <t>(Don't throw out a dollar number yourself, let them quote it, log it, and I'll approve.)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>•  Required: tracked link goat-lab.app/?ref=[code] in [description/bio/pinned comment]; mention it's free</t>
-        </is>
-      </c>
+      <c r="B20" s="17" t="inlineStr"/>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>•  Disclosure: mark it #ad/sponsored (FTC)</t>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>3. Paid-offer terms (after they say yes AND [owner] approves their rate)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>•  Deliverable: [1 dedicated video / 2 posts a week apart / 1 stream segment 20+ min]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>•  Fee: their quoted rate (they name it; [owner] approves before you commit), paid [50% upfront / on posting]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>•  Required: tracked link goat-lab.app/?ref=[code] in [description/bio/pinned comment]; mention it's free</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>•  Disclosure: mark it #ad/sponsored (FTC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>•  Creative control fully theirs; no exclusivity</t>
         </is>
@@ -8554,7 +8578,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>•  Add creators you source yourself to the bottom rows — handle, follower count, sport, and one line on why they fit.</t>
+          <t>•  Add creators you source yourself to the bottom rows: handle, follower count, sport, and one line on why they fit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
marketing: cold DM now signals happy to pay + asks their rate
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/GoatLab-Creator-Tracker.xlsx
+++ b/marketing/GoatLab-Creator-Tracker.xlsx
@@ -8352,7 +8352,7 @@
     <row r="5" ht="15" customHeight="1">
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>Lmk if you'd maybe be interested in making a video/post playing it! No pressure either way.</t>
+          <t>Lmk if you'd be interested in making a video/post playing it! Happy to pay for your time too, just let me know your rate.</t>
         </is>
       </c>
     </row>
@@ -8376,7 +8376,7 @@
     <row r="9" ht="15" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>Lmk if you'd wanna make a video/post on it!</t>
+          <t>Lmk if you'd wanna make a video/post on it! Happy to pay, what's your rate?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
marketing: bump per-1,000 new-players bonus to $15
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/marketing/GoatLab-Creator-Tracker.xlsx
+++ b/marketing/GoatLab-Creator-Tracker.xlsx
@@ -8181,7 +8181,7 @@
     <row r="7" ht="15" customHeight="1">
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>•  $10 for every 1,000 new players your creators send us, each person counted once (not raw plays), tracked through the links (mostly YouTube, X, Twitch).</t>
+          <t>•  $15 for every 1,000 new players your creators send us, each person counted once (not raw plays), tracked through the links (mostly YouTube, X, Twitch).</t>
         </is>
       </c>
     </row>
@@ -8571,7 +8571,7 @@
     <row r="11" ht="15" customHeight="1">
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>•  New players = unique people from the tracking-link report, each counted once no matter how many times they play (ask [owner] for it); drives the $10/1,000 bonus.</t>
+          <t>•  New players = unique people from the tracking-link report, each counted once no matter how many times they play (ask [owner] for it); drives the $15/1,000 bonus.</t>
         </is>
       </c>
     </row>

</xml_diff>